<commit_message>
YHAAO-12383 APM IB - GE_IB_TABLE增加20个字段
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/admin/batchFile/GEIBTableExcel.xlsx
+++ b/src/src/main/webapp/admin/batchFile/GEIBTableExcel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zk\works\codes\hcApmWeb\210408UserAccountType\hc-apm-web\src\src\main\webapp\admin\batchFile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zp\code\web\hc-apm-web-ib\src\src\main\webapp\admin\batchFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07278EB-5194-4429-8CED-2D505F1D2707}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D45327-6766-4AB5-A7D5-1E85C0C4CC29}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>System ID</t>
   </si>
@@ -205,23 +205,83 @@
   <si>
     <t>Sales Pnl</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 st owner-IWIC-手术室</t>
+  </si>
+  <si>
+    <t>1 st owner-IWIC-非手术室</t>
+  </si>
+  <si>
+    <t>1 st owner-OWOC-手术室</t>
+  </si>
+  <si>
+    <t>1 st owner-OWOC-非手术室</t>
+  </si>
+  <si>
+    <t>1 st owner-IWIC-手术室 SSO</t>
+  </si>
+  <si>
+    <t>1 st owner-IWIC-非手术室 SSO</t>
+  </si>
+  <si>
+    <t>1 st owner-OWOC-手术室 SSO</t>
+  </si>
+  <si>
+    <t>1 st owner-OWOC-非手术室 SSO</t>
+  </si>
+  <si>
+    <t>2 nd owner-IWIC-手术室</t>
+  </si>
+  <si>
+    <t>2 nd owner-IWIC-非手术室</t>
+  </si>
+  <si>
+    <t>2 nd owner-OWOC-手术室</t>
+  </si>
+  <si>
+    <t>2 nd owner-OWOC-非手术室</t>
+  </si>
+  <si>
+    <t>2 nd owner-IWIC-手术室 SSO</t>
+  </si>
+  <si>
+    <t>2 nd owner-IWIC-非手术室 SSO</t>
+  </si>
+  <si>
+    <t>2 nd owner-OWOC-手术室 SSO</t>
+  </si>
+  <si>
+    <t>2 nd owner-OWOC-非手术室 SSO</t>
+  </si>
+  <si>
+    <t>SALES_REGION_MGR</t>
+  </si>
+  <si>
+    <t>SALES_REGION_MGR_SSO</t>
+  </si>
+  <si>
+    <t>FE_HEAD_NAME</t>
+  </si>
+  <si>
+    <t>FE_HEAD_SSO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -555,33 +615,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BD1"/>
-  <sheetFormatPr defaultRowHeight="14.1" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:BX1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.44921875" style="5" customWidth="1"/>
-    <col min="19" max="19" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.6484375" customWidth="1"/>
-    <col min="32" max="32" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.44921875" customWidth="1"/>
-    <col min="36" max="36" width="13.75" customWidth="1"/>
-    <col min="37" max="37" width="16.44921875" customWidth="1"/>
-    <col min="38" max="38" width="11.09765625" customWidth="1"/>
-    <col min="44" max="44" width="16.796875" customWidth="1"/>
+    <col min="1" max="1" width="14.41796875" style="5" customWidth="1"/>
+    <col min="19" max="19" width="9.7890625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.62890625" customWidth="1"/>
+    <col min="32" max="32" width="12.26171875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.41796875" customWidth="1"/>
+    <col min="36" max="36" width="13.734375" customWidth="1"/>
+    <col min="37" max="37" width="16.41796875" customWidth="1"/>
+    <col min="38" max="38" width="11.1015625" customWidth="1"/>
+    <col min="44" max="44" width="16.7890625" customWidth="1"/>
     <col min="45" max="45" width="18" customWidth="1"/>
-    <col min="46" max="46" width="15.796875" customWidth="1"/>
-    <col min="47" max="47" width="12.75" customWidth="1"/>
-    <col min="48" max="48" width="14.09765625" customWidth="1"/>
-    <col min="49" max="49" width="12.6484375" customWidth="1"/>
-    <col min="50" max="50" width="13.44921875" customWidth="1"/>
+    <col min="46" max="46" width="15.7890625" customWidth="1"/>
+    <col min="47" max="47" width="12.734375" customWidth="1"/>
+    <col min="48" max="48" width="14.1015625" customWidth="1"/>
+    <col min="49" max="49" width="12.62890625" customWidth="1"/>
+    <col min="50" max="50" width="13.41796875" customWidth="1"/>
     <col min="51" max="51" width="31" customWidth="1"/>
-    <col min="52" max="52" width="18.796875" customWidth="1"/>
-    <col min="53" max="53" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.34765625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="18.7890625" customWidth="1"/>
+    <col min="53" max="53" width="33.47265625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.3671875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="6.26171875" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="10.47265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:76">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -749,6 +809,66 @@
       </c>
       <c r="BD1" s="3" t="s">
         <v>55</v>
+      </c>
+      <c r="BE1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Hc apm web ib gameplan us ibs"
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/admin/batchFile/GEIBTableExcel.xlsx
+++ b/src/src/main/webapp/admin/batchFile/GEIBTableExcel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zk\works\需求\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zk\works\codes\hcApmWeb\210408UserAccountType\hc-apm-web\src\src\main\webapp\admin\batchFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E345E02B-6BDC-4D2E-87E5-6362226F8074}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07278EB-5194-4429-8CED-2D505F1D2707}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>System ID</t>
   </si>
@@ -204,74 +204,6 @@
   </si>
   <si>
     <t>Sales Pnl</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1 st owner-IWIC-手术室</t>
-  </si>
-  <si>
-    <t>1 st owner-IWIC-非手术室</t>
-  </si>
-  <si>
-    <t>1 st owner-OWOC-手术室</t>
-  </si>
-  <si>
-    <t>1 st owner-OWOC-非手术室</t>
-  </si>
-  <si>
-    <t>1 st owner-IWIC-手术室 SSO</t>
-  </si>
-  <si>
-    <t>1 st owner-IWIC-非手术室 SSO</t>
-  </si>
-  <si>
-    <t>1 st owner-OWOC-手术室 SSO</t>
-  </si>
-  <si>
-    <t>1 st owner-OWOC-非手术室 SSO</t>
-  </si>
-  <si>
-    <t>2 nd owner-IWIC-手术室</t>
-  </si>
-  <si>
-    <t>2 nd owner-IWIC-非手术室</t>
-  </si>
-  <si>
-    <t>2 nd owner-OWOC-手术室</t>
-  </si>
-  <si>
-    <t>2 nd owner-OWOC-非手术室</t>
-  </si>
-  <si>
-    <t>2 nd owner-IWIC-手术室 SSO</t>
-  </si>
-  <si>
-    <t>2 nd owner-IWIC-非手术室 SSO</t>
-  </si>
-  <si>
-    <t>2 nd owner-OWOC-手术室 SSO</t>
-  </si>
-  <si>
-    <t>2 nd owner-OWOC-非手术室 SSO</t>
-  </si>
-  <si>
-    <t>SALES_REGION_MGR</t>
-  </si>
-  <si>
-    <t>SALES_REGION_MGR_SSO</t>
-  </si>
-  <si>
-    <t>FE_HEAD_NAME</t>
-  </si>
-  <si>
-    <t>FE_HEAD_SSO</t>
-  </si>
-  <si>
-    <t>Ib Status Present</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>serviceable_ib</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -345,7 +277,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -623,16 +555,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BZ1"/>
+  <dimension ref="A1:BD1"/>
   <sheetFormatPr defaultRowHeight="14.1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="14.3984375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="14.44921875" style="5" customWidth="1"/>
     <col min="19" max="19" width="9.796875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="20.6484375" customWidth="1"/>
     <col min="32" max="32" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.3984375" customWidth="1"/>
+    <col min="35" max="35" width="12.44921875" customWidth="1"/>
     <col min="36" max="36" width="13.75" customWidth="1"/>
-    <col min="37" max="37" width="16.3984375" customWidth="1"/>
+    <col min="37" max="37" width="16.44921875" customWidth="1"/>
     <col min="38" max="38" width="11.09765625" customWidth="1"/>
     <col min="44" max="44" width="16.796875" customWidth="1"/>
     <col min="45" max="45" width="18" customWidth="1"/>
@@ -640,19 +572,16 @@
     <col min="47" max="47" width="12.75" customWidth="1"/>
     <col min="48" max="48" width="14.09765625" customWidth="1"/>
     <col min="49" max="49" width="12.6484375" customWidth="1"/>
-    <col min="50" max="50" width="13.3984375" customWidth="1"/>
+    <col min="50" max="50" width="13.44921875" customWidth="1"/>
     <col min="51" max="51" width="31" customWidth="1"/>
     <col min="52" max="52" width="18.796875" customWidth="1"/>
-    <col min="53" max="53" width="33.44921875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="33.5" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="8.34765625" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="10.44921875" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="12.34765625" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="14.34765625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="14.1484375" customWidth="1"/>
+    <col min="56" max="56" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:78" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.5">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -820,72 +749,6 @@
       </c>
       <c r="BD1" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="BE1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="BF1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="BG1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="BH1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="BI1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="BJ1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="BK1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BL1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="BM1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="BN1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="BO1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="BP1" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="BQ1" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="BR1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="BS1" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="BT1" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BV1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>74</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>75</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>76</v>
-      </c>
-      <c r="BZ1" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>